<commit_message>
Update UK launch date to 6 weeks per confirmed scenario
Sets the UK Restock Plan's launch-date assumption to 2026-09-21
(3 new UK retail partners launching 6 weeks out, per the operations
coordinator scenario), replacing the earlier 8-week placeholder.

With the tighter window, every SKU's sea-freight lead time now
exceeds weeks-to-launch, so all 9 SKUs recalculate to Air — Expedite
(none Critical — air still gets everyone there in time). Total
restock need is unchanged at 4,600 units.
</commit_message>
<xml_diff>
--- a/UK_Restock_Plan.xlsx
+++ b/UK_Restock_Plan.xlsx
@@ -75,7 +75,7 @@
     <t xml:space="preserve">Launch Assumptions (editable):</t>
   </si>
   <si>
-    <t xml:space="preserve">EDIT ME — set actual UK launch date</t>
+    <t xml:space="preserve">3 new UK retail partners launch in 6 weeks (from 2026-08-10) — edit if the date shifts</t>
   </si>
   <si>
     <t xml:space="preserve">Target Weeks of Cover at Launch</t>
@@ -1393,7 +1393,7 @@
       </c>
       <c r="B10" s="6" t="n">
         <f aca="false">'UK Restock Plan'!B4</f>
-        <v>46300</v>
+        <v>46286</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1402,7 +1402,7 @@
       </c>
       <c r="B11" s="7" t="n">
         <f aca="false">'UK Restock Plan'!B7</f>
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1420,7 +1420,7 @@
       </c>
       <c r="B13" s="9" t="n">
         <f aca="false">COUNTIF('UK Restock Plan'!V10:V18,"On Track")</f>
-        <v>8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1429,7 +1429,7 @@
       </c>
       <c r="B14" s="9" t="n">
         <f aca="false">COUNTIF('UK Restock Plan'!V10:V18,"Expedite Required")</f>
-        <v>1</v>
+        <v>9</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1563,7 +1563,7 @@
         <v>4</v>
       </c>
       <c r="B4" s="13" t="n">
-        <v>46300</v>
+        <v>46286</v>
       </c>
       <c r="C4" s="14" t="s">
         <v>16</v>
@@ -1595,7 +1595,7 @@
       </c>
       <c r="B7" s="17" t="n">
         <f aca="false">($B$4-$B$6)/7</f>
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1745,15 +1745,15 @@
       </c>
       <c r="T10" s="22" t="str">
         <f aca="false">IF($N10=0,"No Order Needed",IF($R10&lt;=$B$7,"Sea",IF($S10&lt;=$B$7,"Air — Expedite","Air — Still At Risk")))</f>
-        <v>Sea</v>
+        <v>Air — Expedite</v>
       </c>
       <c r="U10" s="16" t="n">
         <f aca="false">IF($N10=0,"N/A",$B$4-IF($T10="Sea",$R10,$S10)*7)</f>
-        <v>46244</v>
+        <v>46258</v>
       </c>
       <c r="V10" s="22" t="str">
         <f aca="false">IF($N10=0,"No Restock Needed",IF($T10="Sea","On Track",IF($T10="Air — Expedite","Expedite Required","Critical — May Miss Launch")))</f>
-        <v>On Track</v>
+        <v>Expedite Required</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1835,15 +1835,15 @@
       </c>
       <c r="T11" s="22" t="str">
         <f aca="false">IF($N11=0,"No Order Needed",IF($R11&lt;=$B$7,"Sea",IF($S11&lt;=$B$7,"Air — Expedite","Air — Still At Risk")))</f>
-        <v>Sea</v>
+        <v>Air — Expedite</v>
       </c>
       <c r="U11" s="16" t="n">
         <f aca="false">IF($N11=0,"N/A",$B$4-IF($T11="Sea",$R11,$S11)*7)</f>
-        <v>46244</v>
+        <v>46258</v>
       </c>
       <c r="V11" s="22" t="str">
         <f aca="false">IF($N11=0,"No Restock Needed",IF($T11="Sea","On Track",IF($T11="Air — Expedite","Expedite Required","Critical — May Miss Launch")))</f>
-        <v>On Track</v>
+        <v>Expedite Required</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1925,15 +1925,15 @@
       </c>
       <c r="T12" s="22" t="str">
         <f aca="false">IF($N12=0,"No Order Needed",IF($R12&lt;=$B$7,"Sea",IF($S12&lt;=$B$7,"Air — Expedite","Air — Still At Risk")))</f>
-        <v>Sea</v>
+        <v>Air — Expedite</v>
       </c>
       <c r="U12" s="16" t="n">
         <f aca="false">IF($N12=0,"N/A",$B$4-IF($T12="Sea",$R12,$S12)*7)</f>
-        <v>46251</v>
+        <v>46261.5</v>
       </c>
       <c r="V12" s="22" t="str">
         <f aca="false">IF($N12=0,"No Restock Needed",IF($T12="Sea","On Track",IF($T12="Air — Expedite","Expedite Required","Critical — May Miss Launch")))</f>
-        <v>On Track</v>
+        <v>Expedite Required</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2015,15 +2015,15 @@
       </c>
       <c r="T13" s="22" t="str">
         <f aca="false">IF($N13=0,"No Order Needed",IF($R13&lt;=$B$7,"Sea",IF($S13&lt;=$B$7,"Air — Expedite","Air — Still At Risk")))</f>
-        <v>Sea</v>
+        <v>Air — Expedite</v>
       </c>
       <c r="U13" s="16" t="n">
         <f aca="false">IF($N13=0,"N/A",$B$4-IF($T13="Sea",$R13,$S13)*7)</f>
-        <v>46244</v>
+        <v>46258</v>
       </c>
       <c r="V13" s="22" t="str">
         <f aca="false">IF($N13=0,"No Restock Needed",IF($T13="Sea","On Track",IF($T13="Air — Expedite","Expedite Required","Critical — May Miss Launch")))</f>
-        <v>On Track</v>
+        <v>Expedite Required</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2105,15 +2105,15 @@
       </c>
       <c r="T14" s="22" t="str">
         <f aca="false">IF($N14=0,"No Order Needed",IF($R14&lt;=$B$7,"Sea",IF($S14&lt;=$B$7,"Air — Expedite","Air — Still At Risk")))</f>
-        <v>Sea</v>
+        <v>Air — Expedite</v>
       </c>
       <c r="U14" s="16" t="n">
         <f aca="false">IF($N14=0,"N/A",$B$4-IF($T14="Sea",$R14,$S14)*7)</f>
-        <v>46251</v>
+        <v>46266</v>
       </c>
       <c r="V14" s="22" t="str">
         <f aca="false">IF($N14=0,"No Restock Needed",IF($T14="Sea","On Track",IF($T14="Air — Expedite","Expedite Required","Critical — May Miss Launch")))</f>
-        <v>On Track</v>
+        <v>Expedite Required</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2195,15 +2195,15 @@
       </c>
       <c r="T15" s="22" t="str">
         <f aca="false">IF($N15=0,"No Order Needed",IF($R15&lt;=$B$7,"Sea",IF($S15&lt;=$B$7,"Air — Expedite","Air — Still At Risk")))</f>
-        <v>Sea</v>
+        <v>Air — Expedite</v>
       </c>
       <c r="U15" s="16" t="n">
         <f aca="false">IF($N15=0,"N/A",$B$4-IF($T15="Sea",$R15,$S15)*7)</f>
-        <v>46244</v>
+        <v>46258</v>
       </c>
       <c r="V15" s="22" t="str">
         <f aca="false">IF($N15=0,"No Restock Needed",IF($T15="Sea","On Track",IF($T15="Air — Expedite","Expedite Required","Critical — May Miss Launch")))</f>
-        <v>On Track</v>
+        <v>Expedite Required</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2285,15 +2285,15 @@
       </c>
       <c r="T16" s="22" t="str">
         <f aca="false">IF($N16=0,"No Order Needed",IF($R16&lt;=$B$7,"Sea",IF($S16&lt;=$B$7,"Air — Expedite","Air — Still At Risk")))</f>
-        <v>Sea</v>
+        <v>Air — Expedite</v>
       </c>
       <c r="U16" s="16" t="n">
         <f aca="false">IF($N16=0,"N/A",$B$4-IF($T16="Sea",$R16,$S16)*7)</f>
-        <v>46254.5</v>
+        <v>46265</v>
       </c>
       <c r="V16" s="22" t="str">
         <f aca="false">IF($N16=0,"No Restock Needed",IF($T16="Sea","On Track",IF($T16="Air — Expedite","Expedite Required","Critical — May Miss Launch")))</f>
-        <v>On Track</v>
+        <v>Expedite Required</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2379,7 +2379,7 @@
       </c>
       <c r="U17" s="16" t="n">
         <f aca="false">IF($N17=0,"N/A",$B$4-IF($T17="Sea",$R17,$S17)*7)</f>
-        <v>46265</v>
+        <v>46251</v>
       </c>
       <c r="V17" s="22" t="str">
         <f aca="false">IF($N17=0,"No Restock Needed",IF($T17="Sea","On Track",IF($T17="Air — Expedite","Expedite Required","Critical — May Miss Launch")))</f>
@@ -2465,15 +2465,15 @@
       </c>
       <c r="T18" s="22" t="str">
         <f aca="false">IF($N18=0,"No Order Needed",IF($R18&lt;=$B$7,"Sea",IF($S18&lt;=$B$7,"Air — Expedite","Air — Still At Risk")))</f>
-        <v>Sea</v>
+        <v>Air — Expedite</v>
       </c>
       <c r="U18" s="16" t="n">
         <f aca="false">IF($N18=0,"N/A",$B$4-IF($T18="Sea",$R18,$S18)*7)</f>
-        <v>46244</v>
+        <v>46258</v>
       </c>
       <c r="V18" s="22" t="str">
         <f aca="false">IF($N18=0,"No Restock Needed",IF($T18="Sea","On Track",IF($T18="Air — Expedite","Expedite Required","Critical — May Miss Launch")))</f>
-        <v>On Track</v>
+        <v>Expedite Required</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Update restock plan for PO-410 delay and earlier UK launch date
Factory A email: PO-410 (HN-RB-300, 500 units, ships to HK) delayed
2 weeks by a power outage; ETA revised 3.5 -> 5.5 weeks. Status text
updated so it now flags High Risk and surfaces in PO Follow-Ups
(Purchase Order Risk 2 -> 3 High Risk POs). PO-411 (also Factory A)
left unchanged per the factory's confirmation it's unaffected.

Retail partner email: launch date moved up 2 weeks, from 2026-09-21
to 2026-09-07, per their request to confirm stock availability
against the earlier date.

Net effect: weeks until launch drops to ~3.9, and 6 of 9 SKUs now
flag Critical -- May Miss Launch even via air freight (previously 0
were Critical at the 6-week date). Only Body Wash, Lip Balm, and
Essential Oil still make it via expedited air.
</commit_message>
<xml_diff>
--- a/UK_Restock_Plan.xlsx
+++ b/UK_Restock_Plan.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="207">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="208">
   <si>
     <t xml:space="preserve">UK Restock Plan — Summary</t>
   </si>
@@ -81,7 +81,7 @@
     <t xml:space="preserve">Launch Assumptions (editable):</t>
   </si>
   <si>
-    <t xml:space="preserve">3 new UK retail partners launch in 6 weeks (from 2026-08-10) — edit if the date shifts</t>
+    <t xml:space="preserve">UPDATED per retail partner request: moved up 2 weeks from 2026-09-21 (marketing campaign ready early) — was originally 6 weeks out from 2026-08-10</t>
   </si>
   <si>
     <t xml:space="preserve">Target Weeks of Cover at Launch</t>
@@ -308,22 +308,25 @@
     <t xml:space="preserve">HN-RB-300</t>
   </si>
   <si>
+    <t xml:space="preserve">Production delayed — power outage at factory (2-week delay)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sea</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ships to HK, ETA revised to 5.5 weeks (originally 3.5 weeks; +2 weeks for power-outage delay per factory email)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PO-411</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HN-NC-075</t>
+  </si>
+  <si>
     <t xml:space="preserve">In production — on track</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sea</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ships to HK, ETA 3.5 weeks</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PO-411</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HN-NC-075</t>
   </si>
   <si>
     <t xml:space="preserve">US</t>
@@ -1404,7 +1407,7 @@
     <row r="7" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="str">
         <f aca="false">"Purchase Order Risk: "&amp;COUNTIF('Purchase Orders'!O6:O11,"High Risk")&amp;" of "&amp;COUNTA('Purchase Orders'!A6:A11)&amp;" open PO(s) are flagged High Risk and require follow-up."</f>
-        <v>Purchase Order Risk: 2 of 6 open PO(s) are flagged High Risk and require follow-up.</v>
+        <v>Purchase Order Risk: 3 of 6 open PO(s) are flagged High Risk and require follow-up.</v>
       </c>
       <c r="B7" s="4"/>
       <c r="C7" s="4"/>
@@ -1438,7 +1441,7 @@
       </c>
       <c r="B11" s="6" t="n">
         <f aca="false">'UK Restock Plan'!B4</f>
-        <v>46286</v>
+        <v>46272</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1447,7 +1450,7 @@
       </c>
       <c r="B12" s="7" t="n">
         <f aca="false">'UK Restock Plan'!B8</f>
-        <v>5.85714285714286</v>
+        <v>3.85714285714286</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1483,7 +1486,7 @@
       </c>
       <c r="B16" s="9" t="n">
         <f aca="false">COUNTIF('UK Restock Plan'!W11:W19,"Expedite Required")</f>
-        <v>9</v>
+        <v>3</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1492,7 +1495,7 @@
       </c>
       <c r="B17" s="9" t="n">
         <f aca="false">COUNTIF('UK Restock Plan'!W11:W19,"Critical — May Miss Launch")</f>
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1501,7 +1504,7 @@
       </c>
       <c r="B18" s="9" t="n">
         <f aca="false">COUNTIF('PO Follow-Ups'!J6:J11,"Yes")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1635,7 +1638,7 @@
         <v>4</v>
       </c>
       <c r="B4" s="13" t="n">
-        <v>46286</v>
+        <v>46272</v>
       </c>
       <c r="C4" s="14" t="s">
         <v>18</v>
@@ -1678,7 +1681,7 @@
       </c>
       <c r="B8" s="18" t="n">
         <f aca="false">($B$4-$B$7)/7</f>
-        <v>5.85714285714286</v>
+        <v>3.85714285714286</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1834,15 +1837,15 @@
       </c>
       <c r="U11" s="23" t="str">
         <f aca="false">IF($O11=0,"No Order Needed",IF($S11&lt;=$B$8,"Sea",IF($T11&lt;=$B$8,"Air — Expedite","Air — Still At Risk")))</f>
-        <v>Air — Expedite</v>
+        <v>Air — Still At Risk</v>
       </c>
       <c r="V11" s="17" t="n">
         <f aca="false">IF($O11=0,"N/A",$B$4-IF($U11="Sea",$S11,$T11)*7)</f>
-        <v>46258</v>
+        <v>46244</v>
       </c>
       <c r="W11" s="23" t="str">
         <f aca="false">IF($O11=0,"No Restock Needed",IF($U11="Sea","On Track",IF($U11="Air — Expedite","Expedite Required","Critical — May Miss Launch")))</f>
-        <v>Expedite Required</v>
+        <v>Critical — May Miss Launch</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1927,15 +1930,15 @@
       </c>
       <c r="U12" s="23" t="str">
         <f aca="false">IF($O12=0,"No Order Needed",IF($S12&lt;=$B$8,"Sea",IF($T12&lt;=$B$8,"Air — Expedite","Air — Still At Risk")))</f>
-        <v>Air — Expedite</v>
+        <v>Air — Still At Risk</v>
       </c>
       <c r="V12" s="17" t="n">
         <f aca="false">IF($O12=0,"N/A",$B$4-IF($U12="Sea",$S12,$T12)*7)</f>
-        <v>46258</v>
+        <v>46244</v>
       </c>
       <c r="W12" s="23" t="str">
         <f aca="false">IF($O12=0,"No Restock Needed",IF($U12="Sea","On Track",IF($U12="Air — Expedite","Expedite Required","Critical — May Miss Launch")))</f>
-        <v>Expedite Required</v>
+        <v>Critical — May Miss Launch</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2024,7 +2027,7 @@
       </c>
       <c r="V13" s="17" t="n">
         <f aca="false">IF($O13=0,"N/A",$B$4-IF($U13="Sea",$S13,$T13)*7)</f>
-        <v>46261.5</v>
+        <v>46247.5</v>
       </c>
       <c r="W13" s="23" t="str">
         <f aca="false">IF($O13=0,"No Restock Needed",IF($U13="Sea","On Track",IF($U13="Air — Expedite","Expedite Required","Critical — May Miss Launch")))</f>
@@ -2113,15 +2116,15 @@
       </c>
       <c r="U14" s="23" t="str">
         <f aca="false">IF($O14=0,"No Order Needed",IF($S14&lt;=$B$8,"Sea",IF($T14&lt;=$B$8,"Air — Expedite","Air — Still At Risk")))</f>
-        <v>Air — Expedite</v>
+        <v>Air — Still At Risk</v>
       </c>
       <c r="V14" s="17" t="n">
         <f aca="false">IF($O14=0,"N/A",$B$4-IF($U14="Sea",$S14,$T14)*7)</f>
-        <v>46258</v>
+        <v>46244</v>
       </c>
       <c r="W14" s="23" t="str">
         <f aca="false">IF($O14=0,"No Restock Needed",IF($U14="Sea","On Track",IF($U14="Air — Expedite","Expedite Required","Critical — May Miss Launch")))</f>
-        <v>Expedite Required</v>
+        <v>Critical — May Miss Launch</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2210,7 +2213,7 @@
       </c>
       <c r="V15" s="17" t="n">
         <f aca="false">IF($O15=0,"N/A",$B$4-IF($U15="Sea",$S15,$T15)*7)</f>
-        <v>46266</v>
+        <v>46252</v>
       </c>
       <c r="W15" s="23" t="str">
         <f aca="false">IF($O15=0,"No Restock Needed",IF($U15="Sea","On Track",IF($U15="Air — Expedite","Expedite Required","Critical — May Miss Launch")))</f>
@@ -2299,15 +2302,15 @@
       </c>
       <c r="U16" s="23" t="str">
         <f aca="false">IF($O16=0,"No Order Needed",IF($S16&lt;=$B$8,"Sea",IF($T16&lt;=$B$8,"Air — Expedite","Air — Still At Risk")))</f>
-        <v>Air — Expedite</v>
+        <v>Air — Still At Risk</v>
       </c>
       <c r="V16" s="17" t="n">
         <f aca="false">IF($O16=0,"N/A",$B$4-IF($U16="Sea",$S16,$T16)*7)</f>
-        <v>46258</v>
+        <v>46244</v>
       </c>
       <c r="W16" s="23" t="str">
         <f aca="false">IF($O16=0,"No Restock Needed",IF($U16="Sea","On Track",IF($U16="Air — Expedite","Expedite Required","Critical — May Miss Launch")))</f>
-        <v>Expedite Required</v>
+        <v>Critical — May Miss Launch</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2396,7 +2399,7 @@
       </c>
       <c r="V17" s="17" t="n">
         <f aca="false">IF($O17=0,"N/A",$B$4-IF($U17="Sea",$S17,$T17)*7)</f>
-        <v>46265</v>
+        <v>46251</v>
       </c>
       <c r="W17" s="23" t="str">
         <f aca="false">IF($O17=0,"No Restock Needed",IF($U17="Sea","On Track",IF($U17="Air — Expedite","Expedite Required","Critical — May Miss Launch")))</f>
@@ -2485,15 +2488,15 @@
       </c>
       <c r="U18" s="23" t="str">
         <f aca="false">IF($O18=0,"No Order Needed",IF($S18&lt;=$B$8,"Sea",IF($T18&lt;=$B$8,"Air — Expedite","Air — Still At Risk")))</f>
-        <v>Air — Expedite</v>
+        <v>Air — Still At Risk</v>
       </c>
       <c r="V18" s="17" t="n">
         <f aca="false">IF($O18=0,"N/A",$B$4-IF($U18="Sea",$S18,$T18)*7)</f>
-        <v>46251</v>
+        <v>46237</v>
       </c>
       <c r="W18" s="23" t="str">
         <f aca="false">IF($O18=0,"No Restock Needed",IF($U18="Sea","On Track",IF($U18="Air — Expedite","Expedite Required","Critical — May Miss Launch")))</f>
-        <v>Expedite Required</v>
+        <v>Critical — May Miss Launch</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2578,15 +2581,15 @@
       </c>
       <c r="U19" s="23" t="str">
         <f aca="false">IF($O19=0,"No Order Needed",IF($S19&lt;=$B$8,"Sea",IF($T19&lt;=$B$8,"Air — Expedite","Air — Still At Risk")))</f>
-        <v>Air — Expedite</v>
+        <v>Air — Still At Risk</v>
       </c>
       <c r="V19" s="17" t="n">
         <f aca="false">IF($O19=0,"N/A",$B$4-IF($U19="Sea",$S19,$T19)*7)</f>
-        <v>46258</v>
+        <v>46244</v>
       </c>
       <c r="W19" s="23" t="str">
         <f aca="false">IF($O19=0,"No Restock Needed",IF($U19="Sea","On Track",IF($U19="Air — Expedite","Expedite Required","Critical — May Miss Launch")))</f>
-        <v>Expedite Required</v>
+        <v>Critical — May Miss Launch</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2980,11 +2983,11 @@
       </c>
       <c r="F6" s="20" t="str">
         <f aca="false">'Purchase Orders'!G6</f>
-        <v>In production — on track</v>
+        <v>Production delayed — power outage at factory (2-week delay)</v>
       </c>
       <c r="G6" s="23" t="str">
         <f aca="false">'Purchase Orders'!O6</f>
-        <v>Low Risk</v>
+        <v>High Risk</v>
       </c>
       <c r="H6" s="23" t="str">
         <f aca="false">'Purchase Orders'!H6</f>
@@ -2996,15 +2999,15 @@
       </c>
       <c r="J6" s="23" t="str">
         <f aca="false">IF($G6="Low Risk","No","Yes")</f>
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="K6" s="20" t="str">
         <f aca="false">IF(ISNUMBER(SEARCH("delayed",$F6)),"Contact factory for a revised production timeline. If this is a UK-critical SKU, evaluate air freight or a backup factory to recover schedule.",IF(ISNUMBER(SEARCH("Unconfirmed",$F6)),"Escalate to factory immediately — no confirmation received. Confirm the production slot or reallocate the PO to a backup factory.",IF(ISNUMBER(SEARCH("Completed",$F6)),"Issue shipping instructions now. Goods are finished and awaiting dispatch — assign a destination and carrier immediately to avoid storage delays.",IF(ISNUMBER(SEARCH("on track",$F6)),"No follow-up needed — monitor for on-time delivery.","Review PO status manually."))))</f>
-        <v>No follow-up needed — monitor for on-time delivery.</v>
+        <v>Contact factory for a revised production timeline. If this is a UK-critical SKU, evaluate air freight or a backup factory to recover schedule.</v>
       </c>
       <c r="L6" s="23" t="str">
         <f aca="false">IF(AND($G6&lt;&gt;"Low Risk",$I6="Yes — UK Critical SKU"),"Urgent — UK Launch Impact",IF($G6="High Risk","High",IF($G6="Medium Risk","Medium","Low")))</f>
-        <v>Low</v>
+        <v>Urgent — UK Launch Impact</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3514,7 +3517,7 @@
         <v>86</v>
       </c>
       <c r="K6" s="31" t="n">
-        <v>3.5</v>
+        <v>5.5</v>
       </c>
       <c r="L6" s="32" t="n">
         <f aca="false">IFERROR(INDEX('Reference Data'!$C$31:$C$45,MATCH($C6&amp;"|"&amp;$H6,'Reference Data'!$F$31:$F$45,0)),"N/A")</f>
@@ -3530,7 +3533,7 @@
       </c>
       <c r="O6" s="23" t="str">
         <f aca="false">IF(ISNUMBER(SEARCH("delayed",G6)),"High Risk",IF(ISNUMBER(SEARCH("Unconfirmed",G6)),"High Risk",IF(ISNUMBER(SEARCH("Completed",G6)),"Medium Risk",IF(ISNUMBER(SEARCH("on track",G6)),"Low Risk","Review"))))</f>
-        <v>Low Risk</v>
+        <v>High Risk</v>
       </c>
       <c r="P6" s="23" t="str">
         <f aca="false">IF(H6="UK","Yes","No")</f>
@@ -3559,16 +3562,16 @@
         <v>500</v>
       </c>
       <c r="G7" s="28" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="H7" s="30" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="I7" s="30" t="s">
         <v>85</v>
       </c>
       <c r="J7" s="28" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="K7" s="31" t="n">
         <v>4</v>
@@ -3596,17 +3599,17 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="28" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B8" s="28" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C8" s="20" t="str">
         <f aca="false">IFERROR(INDEX('Reference Data'!$B$22:$B$27,MATCH(B8,'Reference Data'!$A$22:$A$27,0)),"N/A")</f>
         <v>Jakarta</v>
       </c>
       <c r="D8" s="28" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="E8" s="20" t="str">
         <f aca="false">IFERROR(INDEX('Reference Data'!$B$10:$B$18,MATCH(D8,'Reference Data'!$A$10:$A$18,0)),"N/A")</f>
@@ -3616,19 +3619,19 @@
         <v>300</v>
       </c>
       <c r="G8" s="28" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="H8" s="30" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I8" s="30" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="J8" s="28" t="s">
+        <v>97</v>
+      </c>
+      <c r="K8" s="30" t="s">
         <v>96</v>
-      </c>
-      <c r="K8" s="30" t="s">
-        <v>95</v>
       </c>
       <c r="L8" s="32" t="str">
         <f aca="false">IFERROR(INDEX('Reference Data'!$C$31:$C$45,MATCH($C8&amp;"|"&amp;$H8,'Reference Data'!$F$31:$F$45,0)),"N/A")</f>
@@ -3653,17 +3656,17 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="28" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B9" s="28" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C9" s="20" t="str">
         <f aca="false">IFERROR(INDEX('Reference Data'!$B$22:$B$27,MATCH(B9,'Reference Data'!$A$22:$A$27,0)),"N/A")</f>
         <v>Taipei</v>
       </c>
       <c r="D9" s="28" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E9" s="20" t="str">
         <f aca="false">IFERROR(INDEX('Reference Data'!$B$10:$B$18,MATCH(D9,'Reference Data'!$A$10:$A$18,0)),"N/A")</f>
@@ -3673,19 +3676,19 @@
         <v>1000</v>
       </c>
       <c r="G9" s="28" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="H9" s="30" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I9" s="30" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="J9" s="28" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="K9" s="30" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="L9" s="32" t="str">
         <f aca="false">IFERROR(INDEX('Reference Data'!$C$31:$C$45,MATCH($C9&amp;"|"&amp;$H9,'Reference Data'!$F$31:$F$45,0)),"N/A")</f>
@@ -3710,17 +3713,17 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="28" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B10" s="28" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C10" s="20" t="str">
         <f aca="false">IFERROR(INDEX('Reference Data'!$B$22:$B$27,MATCH(B10,'Reference Data'!$A$22:$A$27,0)),"N/A")</f>
         <v>Chiang Mai</v>
       </c>
       <c r="D10" s="28" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E10" s="20" t="str">
         <f aca="false">IFERROR(INDEX('Reference Data'!$B$10:$B$18,MATCH(D10,'Reference Data'!$A$10:$A$18,0)),"N/A")</f>
@@ -3730,19 +3733,19 @@
         <v>200</v>
       </c>
       <c r="G10" s="28" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="H10" s="30" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I10" s="30" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="J10" s="28" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="K10" s="30" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="L10" s="32" t="str">
         <f aca="false">IFERROR(INDEX('Reference Data'!$C$31:$C$45,MATCH($C10&amp;"|"&amp;$H10,'Reference Data'!$F$31:$F$45,0)),"N/A")</f>
@@ -3767,17 +3770,17 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="28" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B11" s="28" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C11" s="20" t="str">
         <f aca="false">IFERROR(INDEX('Reference Data'!$B$22:$B$27,MATCH(B11,'Reference Data'!$A$22:$A$27,0)),"N/A")</f>
         <v>Ho Chi Minh City</v>
       </c>
       <c r="D11" s="28" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E11" s="20" t="str">
         <f aca="false">IFERROR(INDEX('Reference Data'!$B$10:$B$18,MATCH(D11,'Reference Data'!$A$10:$A$18,0)),"N/A")</f>
@@ -3787,16 +3790,16 @@
         <v>500</v>
       </c>
       <c r="G11" s="28" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="H11" s="30" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="I11" s="30" t="s">
         <v>85</v>
       </c>
       <c r="J11" s="28" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="K11" s="31" t="n">
         <v>6</v>
@@ -3852,7 +3855,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B15" s="11"/>
       <c r="C15" s="11"/>
@@ -3872,7 +3875,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="11" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B16" s="11"/>
       <c r="C16" s="11"/>
@@ -3892,7 +3895,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="11" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B17" s="11"/>
       <c r="C17" s="11"/>
@@ -3912,7 +3915,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="11" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B18" s="11"/>
       <c r="C18" s="11"/>
@@ -3987,7 +3990,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4006,12 +4009,12 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="12" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B4" s="15" t="n">
         <v>4</v>
@@ -4019,13 +4022,13 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="12" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B5" s="15" t="n">
         <v>8</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4036,40 +4039,40 @@
         <v>25</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D7" s="19" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E7" s="19" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F7" s="19" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="G7" s="19" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="H7" s="19" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="I7" s="19" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="J7" s="19" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="K7" s="19" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="L7" s="19" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="M7" s="19" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="N7" s="19" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="O7" s="19" t="s">
         <v>30</v>
@@ -4134,7 +4137,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="28" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B9" s="20" t="str">
         <f aca="false">IFERROR(INDEX('Reference Data'!$B$10:$B$18,MATCH($A9,'Reference Data'!$A$10:$A$18,0)),"N/A")</f>
@@ -4191,7 +4194,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="28" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B10" s="20" t="str">
         <f aca="false">IFERROR(INDEX('Reference Data'!$B$10:$B$18,MATCH($A10,'Reference Data'!$A$10:$A$18,0)),"N/A")</f>
@@ -4248,7 +4251,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="28" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B11" s="20" t="str">
         <f aca="false">IFERROR(INDEX('Reference Data'!$B$10:$B$18,MATCH($A11,'Reference Data'!$A$10:$A$18,0)),"N/A")</f>
@@ -4305,7 +4308,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="28" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B12" s="20" t="str">
         <f aca="false">IFERROR(INDEX('Reference Data'!$B$10:$B$18,MATCH($A12,'Reference Data'!$A$10:$A$18,0)),"N/A")</f>
@@ -4362,7 +4365,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="28" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B13" s="20" t="str">
         <f aca="false">IFERROR(INDEX('Reference Data'!$B$10:$B$18,MATCH($A13,'Reference Data'!$A$10:$A$18,0)),"N/A")</f>
@@ -4419,7 +4422,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="28" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B14" s="20" t="str">
         <f aca="false">IFERROR(INDEX('Reference Data'!$B$10:$B$18,MATCH($A14,'Reference Data'!$A$10:$A$18,0)),"N/A")</f>
@@ -4476,7 +4479,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="28" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B15" s="20" t="str">
         <f aca="false">IFERROR(INDEX('Reference Data'!$B$10:$B$18,MATCH($A15,'Reference Data'!$A$10:$A$18,0)),"N/A")</f>
@@ -4632,7 +4635,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="11" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B20" s="11"/>
       <c r="C20" s="11"/>
@@ -4651,7 +4654,7 @@
     </row>
     <row r="21" customFormat="false" ht="22.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="11" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B21" s="11"/>
       <c r="C21" s="11"/>
@@ -4670,7 +4673,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="11" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B22" s="11"/>
       <c r="C22" s="11"/>
@@ -4689,7 +4692,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="11" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B23" s="11"/>
       <c r="C23" s="11"/>
@@ -4766,7 +4769,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4778,7 +4781,7 @@
     </row>
     <row r="3" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
@@ -4790,35 +4793,35 @@
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="19" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C4" s="19" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="28" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B5" s="28" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C5" s="28" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="28" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B6" s="28" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C6" s="28" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4826,15 +4829,15 @@
         <v>84</v>
       </c>
       <c r="B7" s="28" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C7" s="28" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
@@ -4852,10 +4855,10 @@
         <v>25</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D9" s="19" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4863,10 +4866,10 @@
         <v>82</v>
       </c>
       <c r="B10" s="28" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C10" s="28" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D10" s="28" t="s">
         <v>81</v>
@@ -4874,13 +4877,13 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="28" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B11" s="28" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C11" s="28" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D11" s="28" t="s">
         <v>81</v>
@@ -4888,86 +4891,86 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="28" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B12" s="28" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C12" s="28" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D12" s="28" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="28" t="s">
+        <v>94</v>
+      </c>
+      <c r="B13" s="28" t="s">
+        <v>158</v>
+      </c>
+      <c r="C13" s="28" t="s">
+        <v>159</v>
+      </c>
+      <c r="D13" s="28" t="s">
         <v>93</v>
-      </c>
-      <c r="B13" s="28" t="s">
-        <v>157</v>
-      </c>
-      <c r="C13" s="28" t="s">
-        <v>158</v>
-      </c>
-      <c r="D13" s="28" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="28" t="s">
+        <v>100</v>
+      </c>
+      <c r="B14" s="28" t="s">
+        <v>160</v>
+      </c>
+      <c r="C14" s="28" t="s">
+        <v>155</v>
+      </c>
+      <c r="D14" s="28" t="s">
         <v>99</v>
-      </c>
-      <c r="B14" s="28" t="s">
-        <v>159</v>
-      </c>
-      <c r="C14" s="28" t="s">
-        <v>154</v>
-      </c>
-      <c r="D14" s="28" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="28" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B15" s="28" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C15" s="28" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D15" s="28" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="28" t="s">
+        <v>105</v>
+      </c>
+      <c r="B16" s="28" t="s">
+        <v>162</v>
+      </c>
+      <c r="C16" s="28" t="s">
+        <v>163</v>
+      </c>
+      <c r="D16" s="28" t="s">
         <v>104</v>
-      </c>
-      <c r="B16" s="28" t="s">
-        <v>161</v>
-      </c>
-      <c r="C16" s="28" t="s">
-        <v>162</v>
-      </c>
-      <c r="D16" s="28" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="28" t="s">
+        <v>109</v>
+      </c>
+      <c r="B17" s="28" t="s">
+        <v>164</v>
+      </c>
+      <c r="C17" s="28" t="s">
+        <v>153</v>
+      </c>
+      <c r="D17" s="28" t="s">
         <v>108</v>
-      </c>
-      <c r="B17" s="28" t="s">
-        <v>163</v>
-      </c>
-      <c r="C17" s="28" t="s">
-        <v>152</v>
-      </c>
-      <c r="D17" s="28" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4975,10 +4978,10 @@
         <v>88</v>
       </c>
       <c r="B18" s="28" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C18" s="28" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D18" s="28" t="s">
         <v>81</v>
@@ -4986,7 +4989,7 @@
     </row>
     <row r="20" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B20" s="3"/>
       <c r="C20" s="3"/>
@@ -5001,22 +5004,22 @@
         <v>26</v>
       </c>
       <c r="B21" s="19" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C21" s="19" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D21" s="19" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="E21" s="19" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="F21" s="19" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="G21" s="19" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="H21" s="19" t="s">
         <v>59</v>
@@ -5027,16 +5030,16 @@
         <v>81</v>
       </c>
       <c r="B22" s="28" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C22" s="28" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D22" s="28" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="E22" s="28" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="F22" s="29" t="n">
         <v>500</v>
@@ -5045,24 +5048,24 @@
         <v>3</v>
       </c>
       <c r="H22" s="28" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="28" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B23" s="28" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C23" s="28" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="D23" s="28" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="E23" s="28" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="F23" s="29" t="n">
         <v>400</v>
@@ -5071,24 +5074,24 @@
         <v>2.5</v>
       </c>
       <c r="H23" s="28" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="28" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B24" s="28" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C24" s="28" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="D24" s="28" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="E24" s="28" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F24" s="29" t="n">
         <v>300</v>
@@ -5097,24 +5100,24 @@
         <v>3</v>
       </c>
       <c r="H24" s="28" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="28" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B25" s="28" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C25" s="28" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D25" s="28" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E25" s="28" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="F25" s="29" t="n">
         <v>1000</v>
@@ -5123,24 +5126,24 @@
         <v>2</v>
       </c>
       <c r="H25" s="28" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="28" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B26" s="28" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C26" s="28" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="D26" s="28" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E26" s="28" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="F26" s="29" t="n">
         <v>200</v>
@@ -5149,24 +5152,24 @@
         <v>2</v>
       </c>
       <c r="H26" s="28" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="28" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B27" s="28" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="C27" s="28" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="D27" s="28" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E27" s="28" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F27" s="29" t="n">
         <v>500</v>
@@ -5175,12 +5178,12 @@
         <v>4</v>
       </c>
       <c r="H27" s="28" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="3" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B29" s="3"/>
       <c r="C29" s="3"/>
@@ -5192,30 +5195,30 @@
     </row>
     <row r="30" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="19" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B30" s="19" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C30" s="19" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="D30" s="19" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="E30" s="19" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="F30" s="19" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="28" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B31" s="28" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C31" s="35" t="n">
         <v>3</v>
@@ -5234,10 +5237,10 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="28" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B32" s="28" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C32" s="35" t="n">
         <v>5</v>
@@ -5256,7 +5259,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="28" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B33" s="28" t="s">
         <v>84</v>
@@ -5278,10 +5281,10 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="28" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B34" s="28" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C34" s="35" t="n">
         <v>4.5</v>
@@ -5300,10 +5303,10 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="28" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B35" s="28" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C35" s="35" t="n">
         <v>4.5</v>
@@ -5322,7 +5325,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="28" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B36" s="28" t="s">
         <v>84</v>
@@ -5344,10 +5347,10 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="28" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B37" s="28" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C37" s="35" t="n">
         <v>4</v>
@@ -5366,10 +5369,10 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="28" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B38" s="28" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C38" s="35" t="n">
         <v>5</v>
@@ -5388,7 +5391,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="28" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B39" s="28" t="s">
         <v>84</v>
@@ -5410,10 +5413,10 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="28" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B40" s="28" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C40" s="35" t="n">
         <v>3</v>
@@ -5432,10 +5435,10 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="28" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B41" s="28" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C41" s="35" t="n">
         <v>5</v>
@@ -5454,7 +5457,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="28" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B42" s="28" t="s">
         <v>84</v>
@@ -5476,10 +5479,10 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="28" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B43" s="28" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C43" s="35" t="n">
         <v>3.5</v>
@@ -5498,10 +5501,10 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="28" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B44" s="28" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C44" s="35" t="n">
         <v>5</v>
@@ -5520,7 +5523,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="28" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B45" s="28" t="s">
         <v>84</v>
@@ -5547,7 +5550,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="11" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B48" s="11"/>
       <c r="C48" s="11"/>
@@ -5559,7 +5562,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="11" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B49" s="11"/>
       <c r="C49" s="11"/>
@@ -5571,7 +5574,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="11" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B50" s="11"/>
       <c r="C50" s="11"/>
@@ -5583,7 +5586,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="11" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B51" s="11"/>
       <c r="C51" s="11"/>
@@ -5595,7 +5598,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="11" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B52" s="11"/>
       <c r="C52" s="11"/>

</xml_diff>

<commit_message>
Add UK shipping days alongside weeks in restock plan
Sea Transit to UK and Air Transit to UK now each show both a Weeks
column and a Days column (Weeks x 7) on the UK Restock Plan tab, per
user request, for day-level shipping planning.

Also adds CLAUDE.md recording this as a standing convention so future
regenerations of the restock plan keep both columns.
</commit_message>
<xml_diff>
--- a/UK_Restock_Plan.xlsx
+++ b/UK_Restock_Plan.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="208">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="327" uniqueCount="211">
   <si>
     <t xml:space="preserve">UK Restock Plan — Summary</t>
   </si>
@@ -166,10 +166,18 @@
 to UK (Wks)</t>
   </si>
   <si>
+    <t xml:space="preserve">Sea Transit
+to UK (Days)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Air Transit
 to UK (Wks)</t>
   </si>
   <si>
+    <t xml:space="preserve">Air Transit
+to UK (Days)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Total Lead
 Time — Sea</t>
   </si>
@@ -206,6 +214,9 @@
   </si>
   <si>
     <t xml:space="preserve">• Recommended Ship Method / Launch Readiness compare each lead-time option (Production Lead Time + Sea or Air transit to UK) against Weeks Until Launch: Sea if it fits, Air if only Air fits, otherwise flagged Critical even with Air.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Sea/Air Transit to UK are shown in both weeks and days (Days = Weeks × 7) per standing instruction, so shipping windows can be planned at day-level precision, not just whole weeks.</t>
   </si>
   <si>
     <t xml:space="preserve">• Order-By Date = Launch Date minus the recommended method's total lead time. If this date is already in the past, that order is overdue and should be placed immediately.</t>
@@ -1476,7 +1487,7 @@
         <v>8</v>
       </c>
       <c r="B15" s="9" t="n">
-        <f aca="false">COUNTIF('UK Restock Plan'!W11:W19,"On Track")</f>
+        <f aca="false">COUNTIF('UK Restock Plan'!Y11:Y19,"On Track")</f>
         <v>0</v>
       </c>
     </row>
@@ -1485,7 +1496,7 @@
         <v>9</v>
       </c>
       <c r="B16" s="9" t="n">
-        <f aca="false">COUNTIF('UK Restock Plan'!W11:W19,"Expedite Required")</f>
+        <f aca="false">COUNTIF('UK Restock Plan'!Y11:Y19,"Expedite Required")</f>
         <v>3</v>
       </c>
     </row>
@@ -1494,7 +1505,7 @@
         <v>10</v>
       </c>
       <c r="B17" s="9" t="n">
-        <f aca="false">COUNTIF('UK Restock Plan'!W11:W19,"Critical — May Miss Launch")</f>
+        <f aca="false">COUNTIF('UK Restock Plan'!Y11:Y19,"Critical — May Miss Launch")</f>
         <v>6</v>
       </c>
     </row>
@@ -1579,7 +1590,7 @@
     <tabColor rgb="FFC00000"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:W29"/>
+  <dimension ref="A1:Y30"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11"/>
@@ -1594,11 +1605,11 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="10"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="16" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="19" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="0" width="17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="23" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="16" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="21" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="23" style="0" width="17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="24" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="25" style="0" width="20"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1627,6 +1638,8 @@
       <c r="U1" s="1"/>
       <c r="V1" s="1"/>
       <c r="W1" s="1"/>
+      <c r="X1" s="1"/>
+      <c r="Y1" s="1"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
@@ -1753,6 +1766,12 @@
       </c>
       <c r="W10" s="19" t="s">
         <v>46</v>
+      </c>
+      <c r="X10" s="19" t="s">
+        <v>47</v>
+      </c>
+      <c r="Y10" s="19" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1823,28 +1842,36 @@
         <f aca="false">IFERROR(INDEX('Reference Data'!$C$31:$C$45,MATCH($D11&amp;"|UK",'Reference Data'!$F$31:$F$45,0)),"N/A")</f>
         <v>5</v>
       </c>
-      <c r="R11" s="25" t="n">
+      <c r="R11" s="22" t="n">
+        <f aca="false">IFERROR($Q11*7,"N/A")</f>
+        <v>35</v>
+      </c>
+      <c r="S11" s="25" t="n">
         <f aca="false">IFERROR(INDEX('Reference Data'!$E$31:$E$45,MATCH($D11&amp;"|UK",'Reference Data'!$F$31:$F$45,0)),"N/A")</f>
         <v>1</v>
       </c>
-      <c r="S11" s="25" t="n">
+      <c r="T11" s="22" t="n">
+        <f aca="false">IFERROR($S11*7,"N/A")</f>
+        <v>7</v>
+      </c>
+      <c r="U11" s="25" t="n">
         <f aca="false">$P11+$Q11</f>
         <v>8</v>
       </c>
-      <c r="T11" s="25" t="n">
-        <f aca="false">$P11+$R11</f>
+      <c r="V11" s="25" t="n">
+        <f aca="false">$P11+$S11</f>
         <v>4</v>
       </c>
-      <c r="U11" s="23" t="str">
-        <f aca="false">IF($O11=0,"No Order Needed",IF($S11&lt;=$B$8,"Sea",IF($T11&lt;=$B$8,"Air — Expedite","Air — Still At Risk")))</f>
+      <c r="W11" s="23" t="str">
+        <f aca="false">IF($O11=0,"No Order Needed",IF($U11&lt;=$B$8,"Sea",IF($V11&lt;=$B$8,"Air — Expedite","Air — Still At Risk")))</f>
         <v>Air — Still At Risk</v>
       </c>
-      <c r="V11" s="17" t="n">
-        <f aca="false">IF($O11=0,"N/A",$B$4-IF($U11="Sea",$S11,$T11)*7)</f>
+      <c r="X11" s="17" t="n">
+        <f aca="false">IF($O11=0,"N/A",$B$4-IF($W11="Sea",$U11,$V11)*7)</f>
         <v>46244</v>
       </c>
-      <c r="W11" s="23" t="str">
-        <f aca="false">IF($O11=0,"No Restock Needed",IF($U11="Sea","On Track",IF($U11="Air — Expedite","Expedite Required","Critical — May Miss Launch")))</f>
+      <c r="Y11" s="23" t="str">
+        <f aca="false">IF($O11=0,"No Restock Needed",IF($W11="Sea","On Track",IF($W11="Air — Expedite","Expedite Required","Critical — May Miss Launch")))</f>
         <v>Critical — May Miss Launch</v>
       </c>
     </row>
@@ -1916,28 +1943,36 @@
         <f aca="false">IFERROR(INDEX('Reference Data'!$C$31:$C$45,MATCH($D12&amp;"|UK",'Reference Data'!$F$31:$F$45,0)),"N/A")</f>
         <v>5</v>
       </c>
-      <c r="R12" s="25" t="n">
+      <c r="R12" s="22" t="n">
+        <f aca="false">IFERROR($Q12*7,"N/A")</f>
+        <v>35</v>
+      </c>
+      <c r="S12" s="25" t="n">
         <f aca="false">IFERROR(INDEX('Reference Data'!$E$31:$E$45,MATCH($D12&amp;"|UK",'Reference Data'!$F$31:$F$45,0)),"N/A")</f>
         <v>1</v>
       </c>
-      <c r="S12" s="25" t="n">
+      <c r="T12" s="22" t="n">
+        <f aca="false">IFERROR($S12*7,"N/A")</f>
+        <v>7</v>
+      </c>
+      <c r="U12" s="25" t="n">
         <f aca="false">$P12+$Q12</f>
         <v>8</v>
       </c>
-      <c r="T12" s="25" t="n">
-        <f aca="false">$P12+$R12</f>
+      <c r="V12" s="25" t="n">
+        <f aca="false">$P12+$S12</f>
         <v>4</v>
       </c>
-      <c r="U12" s="23" t="str">
-        <f aca="false">IF($O12=0,"No Order Needed",IF($S12&lt;=$B$8,"Sea",IF($T12&lt;=$B$8,"Air — Expedite","Air — Still At Risk")))</f>
+      <c r="W12" s="23" t="str">
+        <f aca="false">IF($O12=0,"No Order Needed",IF($U12&lt;=$B$8,"Sea",IF($V12&lt;=$B$8,"Air — Expedite","Air — Still At Risk")))</f>
         <v>Air — Still At Risk</v>
       </c>
-      <c r="V12" s="17" t="n">
-        <f aca="false">IF($O12=0,"N/A",$B$4-IF($U12="Sea",$S12,$T12)*7)</f>
+      <c r="X12" s="17" t="n">
+        <f aca="false">IF($O12=0,"N/A",$B$4-IF($W12="Sea",$U12,$V12)*7)</f>
         <v>46244</v>
       </c>
-      <c r="W12" s="23" t="str">
-        <f aca="false">IF($O12=0,"No Restock Needed",IF($U12="Sea","On Track",IF($U12="Air — Expedite","Expedite Required","Critical — May Miss Launch")))</f>
+      <c r="Y12" s="23" t="str">
+        <f aca="false">IF($O12=0,"No Restock Needed",IF($W12="Sea","On Track",IF($W12="Air — Expedite","Expedite Required","Critical — May Miss Launch")))</f>
         <v>Critical — May Miss Launch</v>
       </c>
     </row>
@@ -2009,28 +2044,36 @@
         <f aca="false">IFERROR(INDEX('Reference Data'!$C$31:$C$45,MATCH($D13&amp;"|UK",'Reference Data'!$F$31:$F$45,0)),"N/A")</f>
         <v>4.5</v>
       </c>
-      <c r="R13" s="25" t="n">
+      <c r="R13" s="22" t="n">
+        <f aca="false">IFERROR($Q13*7,"N/A")</f>
+        <v>31.5</v>
+      </c>
+      <c r="S13" s="25" t="n">
         <f aca="false">IFERROR(INDEX('Reference Data'!$E$31:$E$45,MATCH($D13&amp;"|UK",'Reference Data'!$F$31:$F$45,0)),"N/A")</f>
         <v>1</v>
       </c>
-      <c r="S13" s="25" t="n">
+      <c r="T13" s="22" t="n">
+        <f aca="false">IFERROR($S13*7,"N/A")</f>
+        <v>7</v>
+      </c>
+      <c r="U13" s="25" t="n">
         <f aca="false">$P13+$Q13</f>
         <v>7</v>
       </c>
-      <c r="T13" s="25" t="n">
-        <f aca="false">$P13+$R13</f>
+      <c r="V13" s="25" t="n">
+        <f aca="false">$P13+$S13</f>
         <v>3.5</v>
       </c>
-      <c r="U13" s="23" t="str">
-        <f aca="false">IF($O13=0,"No Order Needed",IF($S13&lt;=$B$8,"Sea",IF($T13&lt;=$B$8,"Air — Expedite","Air — Still At Risk")))</f>
+      <c r="W13" s="23" t="str">
+        <f aca="false">IF($O13=0,"No Order Needed",IF($U13&lt;=$B$8,"Sea",IF($V13&lt;=$B$8,"Air — Expedite","Air — Still At Risk")))</f>
         <v>Air — Expedite</v>
       </c>
-      <c r="V13" s="17" t="n">
-        <f aca="false">IF($O13=0,"N/A",$B$4-IF($U13="Sea",$S13,$T13)*7)</f>
+      <c r="X13" s="17" t="n">
+        <f aca="false">IF($O13=0,"N/A",$B$4-IF($W13="Sea",$U13,$V13)*7)</f>
         <v>46247.5</v>
       </c>
-      <c r="W13" s="23" t="str">
-        <f aca="false">IF($O13=0,"No Restock Needed",IF($U13="Sea","On Track",IF($U13="Air — Expedite","Expedite Required","Critical — May Miss Launch")))</f>
+      <c r="Y13" s="23" t="str">
+        <f aca="false">IF($O13=0,"No Restock Needed",IF($W13="Sea","On Track",IF($W13="Air — Expedite","Expedite Required","Critical — May Miss Launch")))</f>
         <v>Expedite Required</v>
       </c>
     </row>
@@ -2102,28 +2145,36 @@
         <f aca="false">IFERROR(INDEX('Reference Data'!$C$31:$C$45,MATCH($D14&amp;"|UK",'Reference Data'!$F$31:$F$45,0)),"N/A")</f>
         <v>5</v>
       </c>
-      <c r="R14" s="25" t="n">
+      <c r="R14" s="22" t="n">
+        <f aca="false">IFERROR($Q14*7,"N/A")</f>
+        <v>35</v>
+      </c>
+      <c r="S14" s="25" t="n">
         <f aca="false">IFERROR(INDEX('Reference Data'!$E$31:$E$45,MATCH($D14&amp;"|UK",'Reference Data'!$F$31:$F$45,0)),"N/A")</f>
         <v>1</v>
       </c>
-      <c r="S14" s="25" t="n">
+      <c r="T14" s="22" t="n">
+        <f aca="false">IFERROR($S14*7,"N/A")</f>
+        <v>7</v>
+      </c>
+      <c r="U14" s="25" t="n">
         <f aca="false">$P14+$Q14</f>
         <v>8</v>
       </c>
-      <c r="T14" s="25" t="n">
-        <f aca="false">$P14+$R14</f>
+      <c r="V14" s="25" t="n">
+        <f aca="false">$P14+$S14</f>
         <v>4</v>
       </c>
-      <c r="U14" s="23" t="str">
-        <f aca="false">IF($O14=0,"No Order Needed",IF($S14&lt;=$B$8,"Sea",IF($T14&lt;=$B$8,"Air — Expedite","Air — Still At Risk")))</f>
+      <c r="W14" s="23" t="str">
+        <f aca="false">IF($O14=0,"No Order Needed",IF($U14&lt;=$B$8,"Sea",IF($V14&lt;=$B$8,"Air — Expedite","Air — Still At Risk")))</f>
         <v>Air — Still At Risk</v>
       </c>
-      <c r="V14" s="17" t="n">
-        <f aca="false">IF($O14=0,"N/A",$B$4-IF($U14="Sea",$S14,$T14)*7)</f>
+      <c r="X14" s="17" t="n">
+        <f aca="false">IF($O14=0,"N/A",$B$4-IF($W14="Sea",$U14,$V14)*7)</f>
         <v>46244</v>
       </c>
-      <c r="W14" s="23" t="str">
-        <f aca="false">IF($O14=0,"No Restock Needed",IF($U14="Sea","On Track",IF($U14="Air — Expedite","Expedite Required","Critical — May Miss Launch")))</f>
+      <c r="Y14" s="23" t="str">
+        <f aca="false">IF($O14=0,"No Restock Needed",IF($W14="Sea","On Track",IF($W14="Air — Expedite","Expedite Required","Critical — May Miss Launch")))</f>
         <v>Critical — May Miss Launch</v>
       </c>
     </row>
@@ -2195,28 +2246,36 @@
         <f aca="false">IFERROR(INDEX('Reference Data'!$C$31:$C$45,MATCH($D15&amp;"|UK",'Reference Data'!$F$31:$F$45,0)),"N/A")</f>
         <v>5</v>
       </c>
-      <c r="R15" s="25" t="n">
+      <c r="R15" s="22" t="n">
+        <f aca="false">IFERROR($Q15*7,"N/A")</f>
+        <v>35</v>
+      </c>
+      <c r="S15" s="25" t="n">
         <f aca="false">IFERROR(INDEX('Reference Data'!$E$31:$E$45,MATCH($D15&amp;"|UK",'Reference Data'!$F$31:$F$45,0)),"N/A")</f>
         <v>0.857142857142857</v>
       </c>
-      <c r="S15" s="25" t="n">
+      <c r="T15" s="22" t="n">
+        <f aca="false">IFERROR($S15*7,"N/A")</f>
+        <v>6</v>
+      </c>
+      <c r="U15" s="25" t="n">
         <f aca="false">$P15+$Q15</f>
         <v>7</v>
       </c>
-      <c r="T15" s="25" t="n">
-        <f aca="false">$P15+$R15</f>
+      <c r="V15" s="25" t="n">
+        <f aca="false">$P15+$S15</f>
         <v>2.85714285714286</v>
       </c>
-      <c r="U15" s="23" t="str">
-        <f aca="false">IF($O15=0,"No Order Needed",IF($S15&lt;=$B$8,"Sea",IF($T15&lt;=$B$8,"Air — Expedite","Air — Still At Risk")))</f>
+      <c r="W15" s="23" t="str">
+        <f aca="false">IF($O15=0,"No Order Needed",IF($U15&lt;=$B$8,"Sea",IF($V15&lt;=$B$8,"Air — Expedite","Air — Still At Risk")))</f>
         <v>Air — Expedite</v>
       </c>
-      <c r="V15" s="17" t="n">
-        <f aca="false">IF($O15=0,"N/A",$B$4-IF($U15="Sea",$S15,$T15)*7)</f>
+      <c r="X15" s="17" t="n">
+        <f aca="false">IF($O15=0,"N/A",$B$4-IF($W15="Sea",$U15,$V15)*7)</f>
         <v>46252</v>
       </c>
-      <c r="W15" s="23" t="str">
-        <f aca="false">IF($O15=0,"No Restock Needed",IF($U15="Sea","On Track",IF($U15="Air — Expedite","Expedite Required","Critical — May Miss Launch")))</f>
+      <c r="Y15" s="23" t="str">
+        <f aca="false">IF($O15=0,"No Restock Needed",IF($W15="Sea","On Track",IF($W15="Air — Expedite","Expedite Required","Critical — May Miss Launch")))</f>
         <v>Expedite Required</v>
       </c>
     </row>
@@ -2288,28 +2347,36 @@
         <f aca="false">IFERROR(INDEX('Reference Data'!$C$31:$C$45,MATCH($D16&amp;"|UK",'Reference Data'!$F$31:$F$45,0)),"N/A")</f>
         <v>5</v>
       </c>
-      <c r="R16" s="25" t="n">
+      <c r="R16" s="22" t="n">
+        <f aca="false">IFERROR($Q16*7,"N/A")</f>
+        <v>35</v>
+      </c>
+      <c r="S16" s="25" t="n">
         <f aca="false">IFERROR(INDEX('Reference Data'!$E$31:$E$45,MATCH($D16&amp;"|UK",'Reference Data'!$F$31:$F$45,0)),"N/A")</f>
         <v>1</v>
       </c>
-      <c r="S16" s="25" t="n">
+      <c r="T16" s="22" t="n">
+        <f aca="false">IFERROR($S16*7,"N/A")</f>
+        <v>7</v>
+      </c>
+      <c r="U16" s="25" t="n">
         <f aca="false">$P16+$Q16</f>
         <v>8</v>
       </c>
-      <c r="T16" s="25" t="n">
-        <f aca="false">$P16+$R16</f>
+      <c r="V16" s="25" t="n">
+        <f aca="false">$P16+$S16</f>
         <v>4</v>
       </c>
-      <c r="U16" s="23" t="str">
-        <f aca="false">IF($O16=0,"No Order Needed",IF($S16&lt;=$B$8,"Sea",IF($T16&lt;=$B$8,"Air — Expedite","Air — Still At Risk")))</f>
+      <c r="W16" s="23" t="str">
+        <f aca="false">IF($O16=0,"No Order Needed",IF($U16&lt;=$B$8,"Sea",IF($V16&lt;=$B$8,"Air — Expedite","Air — Still At Risk")))</f>
         <v>Air — Still At Risk</v>
       </c>
-      <c r="V16" s="17" t="n">
-        <f aca="false">IF($O16=0,"N/A",$B$4-IF($U16="Sea",$S16,$T16)*7)</f>
+      <c r="X16" s="17" t="n">
+        <f aca="false">IF($O16=0,"N/A",$B$4-IF($W16="Sea",$U16,$V16)*7)</f>
         <v>46244</v>
       </c>
-      <c r="W16" s="23" t="str">
-        <f aca="false">IF($O16=0,"No Restock Needed",IF($U16="Sea","On Track",IF($U16="Air — Expedite","Expedite Required","Critical — May Miss Launch")))</f>
+      <c r="Y16" s="23" t="str">
+        <f aca="false">IF($O16=0,"No Restock Needed",IF($W16="Sea","On Track",IF($W16="Air — Expedite","Expedite Required","Critical — May Miss Launch")))</f>
         <v>Critical — May Miss Launch</v>
       </c>
     </row>
@@ -2381,28 +2448,36 @@
         <f aca="false">IFERROR(INDEX('Reference Data'!$C$31:$C$45,MATCH($D17&amp;"|UK",'Reference Data'!$F$31:$F$45,0)),"N/A")</f>
         <v>4.5</v>
       </c>
-      <c r="R17" s="25" t="n">
+      <c r="R17" s="22" t="n">
+        <f aca="false">IFERROR($Q17*7,"N/A")</f>
+        <v>31.5</v>
+      </c>
+      <c r="S17" s="25" t="n">
         <f aca="false">IFERROR(INDEX('Reference Data'!$E$31:$E$45,MATCH($D17&amp;"|UK",'Reference Data'!$F$31:$F$45,0)),"N/A")</f>
         <v>1</v>
       </c>
-      <c r="S17" s="25" t="n">
+      <c r="T17" s="22" t="n">
+        <f aca="false">IFERROR($S17*7,"N/A")</f>
+        <v>7</v>
+      </c>
+      <c r="U17" s="25" t="n">
         <f aca="false">$P17+$Q17</f>
         <v>6.5</v>
       </c>
-      <c r="T17" s="25" t="n">
-        <f aca="false">$P17+$R17</f>
+      <c r="V17" s="25" t="n">
+        <f aca="false">$P17+$S17</f>
         <v>3</v>
       </c>
-      <c r="U17" s="23" t="str">
-        <f aca="false">IF($O17=0,"No Order Needed",IF($S17&lt;=$B$8,"Sea",IF($T17&lt;=$B$8,"Air — Expedite","Air — Still At Risk")))</f>
+      <c r="W17" s="23" t="str">
+        <f aca="false">IF($O17=0,"No Order Needed",IF($U17&lt;=$B$8,"Sea",IF($V17&lt;=$B$8,"Air — Expedite","Air — Still At Risk")))</f>
         <v>Air — Expedite</v>
       </c>
-      <c r="V17" s="17" t="n">
-        <f aca="false">IF($O17=0,"N/A",$B$4-IF($U17="Sea",$S17,$T17)*7)</f>
+      <c r="X17" s="17" t="n">
+        <f aca="false">IF($O17=0,"N/A",$B$4-IF($W17="Sea",$U17,$V17)*7)</f>
         <v>46251</v>
       </c>
-      <c r="W17" s="23" t="str">
-        <f aca="false">IF($O17=0,"No Restock Needed",IF($U17="Sea","On Track",IF($U17="Air — Expedite","Expedite Required","Critical — May Miss Launch")))</f>
+      <c r="Y17" s="23" t="str">
+        <f aca="false">IF($O17=0,"No Restock Needed",IF($W17="Sea","On Track",IF($W17="Air — Expedite","Expedite Required","Critical — May Miss Launch")))</f>
         <v>Expedite Required</v>
       </c>
     </row>
@@ -2474,28 +2549,36 @@
         <f aca="false">IFERROR(INDEX('Reference Data'!$C$31:$C$45,MATCH($D18&amp;"|UK",'Reference Data'!$F$31:$F$45,0)),"N/A")</f>
         <v>5</v>
       </c>
-      <c r="R18" s="25" t="n">
+      <c r="R18" s="22" t="n">
+        <f aca="false">IFERROR($Q18*7,"N/A")</f>
+        <v>35</v>
+      </c>
+      <c r="S18" s="25" t="n">
         <f aca="false">IFERROR(INDEX('Reference Data'!$E$31:$E$45,MATCH($D18&amp;"|UK",'Reference Data'!$F$31:$F$45,0)),"N/A")</f>
         <v>1</v>
       </c>
-      <c r="S18" s="25" t="n">
+      <c r="T18" s="22" t="n">
+        <f aca="false">IFERROR($S18*7,"N/A")</f>
+        <v>7</v>
+      </c>
+      <c r="U18" s="25" t="n">
         <f aca="false">$P18+$Q18</f>
         <v>9</v>
       </c>
-      <c r="T18" s="25" t="n">
-        <f aca="false">$P18+$R18</f>
+      <c r="V18" s="25" t="n">
+        <f aca="false">$P18+$S18</f>
         <v>5</v>
       </c>
-      <c r="U18" s="23" t="str">
-        <f aca="false">IF($O18=0,"No Order Needed",IF($S18&lt;=$B$8,"Sea",IF($T18&lt;=$B$8,"Air — Expedite","Air — Still At Risk")))</f>
+      <c r="W18" s="23" t="str">
+        <f aca="false">IF($O18=0,"No Order Needed",IF($U18&lt;=$B$8,"Sea",IF($V18&lt;=$B$8,"Air — Expedite","Air — Still At Risk")))</f>
         <v>Air — Still At Risk</v>
       </c>
-      <c r="V18" s="17" t="n">
-        <f aca="false">IF($O18=0,"N/A",$B$4-IF($U18="Sea",$S18,$T18)*7)</f>
+      <c r="X18" s="17" t="n">
+        <f aca="false">IF($O18=0,"N/A",$B$4-IF($W18="Sea",$U18,$V18)*7)</f>
         <v>46237</v>
       </c>
-      <c r="W18" s="23" t="str">
-        <f aca="false">IF($O18=0,"No Restock Needed",IF($U18="Sea","On Track",IF($U18="Air — Expedite","Expedite Required","Critical — May Miss Launch")))</f>
+      <c r="Y18" s="23" t="str">
+        <f aca="false">IF($O18=0,"No Restock Needed",IF($W18="Sea","On Track",IF($W18="Air — Expedite","Expedite Required","Critical — May Miss Launch")))</f>
         <v>Critical — May Miss Launch</v>
       </c>
     </row>
@@ -2567,34 +2650,42 @@
         <f aca="false">IFERROR(INDEX('Reference Data'!$C$31:$C$45,MATCH($D19&amp;"|UK",'Reference Data'!$F$31:$F$45,0)),"N/A")</f>
         <v>5</v>
       </c>
-      <c r="R19" s="25" t="n">
+      <c r="R19" s="22" t="n">
+        <f aca="false">IFERROR($Q19*7,"N/A")</f>
+        <v>35</v>
+      </c>
+      <c r="S19" s="25" t="n">
         <f aca="false">IFERROR(INDEX('Reference Data'!$E$31:$E$45,MATCH($D19&amp;"|UK",'Reference Data'!$F$31:$F$45,0)),"N/A")</f>
         <v>1</v>
       </c>
-      <c r="S19" s="25" t="n">
+      <c r="T19" s="22" t="n">
+        <f aca="false">IFERROR($S19*7,"N/A")</f>
+        <v>7</v>
+      </c>
+      <c r="U19" s="25" t="n">
         <f aca="false">$P19+$Q19</f>
         <v>8</v>
       </c>
-      <c r="T19" s="25" t="n">
-        <f aca="false">$P19+$R19</f>
+      <c r="V19" s="25" t="n">
+        <f aca="false">$P19+$S19</f>
         <v>4</v>
       </c>
-      <c r="U19" s="23" t="str">
-        <f aca="false">IF($O19=0,"No Order Needed",IF($S19&lt;=$B$8,"Sea",IF($T19&lt;=$B$8,"Air — Expedite","Air — Still At Risk")))</f>
+      <c r="W19" s="23" t="str">
+        <f aca="false">IF($O19=0,"No Order Needed",IF($U19&lt;=$B$8,"Sea",IF($V19&lt;=$B$8,"Air — Expedite","Air — Still At Risk")))</f>
         <v>Air — Still At Risk</v>
       </c>
-      <c r="V19" s="17" t="n">
-        <f aca="false">IF($O19=0,"N/A",$B$4-IF($U19="Sea",$S19,$T19)*7)</f>
+      <c r="X19" s="17" t="n">
+        <f aca="false">IF($O19=0,"N/A",$B$4-IF($W19="Sea",$U19,$V19)*7)</f>
         <v>46244</v>
       </c>
-      <c r="W19" s="23" t="str">
-        <f aca="false">IF($O19=0,"No Restock Needed",IF($U19="Sea","On Track",IF($U19="Air — Expedite","Expedite Required","Critical — May Miss Launch")))</f>
+      <c r="Y19" s="23" t="str">
+        <f aca="false">IF($O19=0,"No Restock Needed",IF($W19="Sea","On Track",IF($W19="Air — Expedite","Expedite Required","Critical — May Miss Launch")))</f>
         <v>Critical — May Miss Launch</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="26" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B20" s="27"/>
       <c r="C20" s="27"/>
@@ -2624,6 +2715,8 @@
       <c r="U20" s="27"/>
       <c r="V20" s="27"/>
       <c r="W20" s="27"/>
+      <c r="X20" s="27"/>
+      <c r="Y20" s="27"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="10" t="s">
@@ -2632,7 +2725,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="11" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B23" s="11"/>
       <c r="C23" s="11"/>
@@ -2656,10 +2749,12 @@
       <c r="U23" s="11"/>
       <c r="V23" s="11"/>
       <c r="W23" s="11"/>
+      <c r="X23" s="11"/>
+      <c r="Y23" s="11"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="11" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B24" s="11"/>
       <c r="C24" s="11"/>
@@ -2683,10 +2778,12 @@
       <c r="U24" s="11"/>
       <c r="V24" s="11"/>
       <c r="W24" s="11"/>
+      <c r="X24" s="11"/>
+      <c r="Y24" s="11"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="11" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B25" s="11"/>
       <c r="C25" s="11"/>
@@ -2710,10 +2807,12 @@
       <c r="U25" s="11"/>
       <c r="V25" s="11"/>
       <c r="W25" s="11"/>
+      <c r="X25" s="11"/>
+      <c r="Y25" s="11"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="11" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B26" s="11"/>
       <c r="C26" s="11"/>
@@ -2737,10 +2836,12 @@
       <c r="U26" s="11"/>
       <c r="V26" s="11"/>
       <c r="W26" s="11"/>
+      <c r="X26" s="11"/>
+      <c r="Y26" s="11"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="11" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B27" s="11"/>
       <c r="C27" s="11"/>
@@ -2764,10 +2865,12 @@
       <c r="U27" s="11"/>
       <c r="V27" s="11"/>
       <c r="W27" s="11"/>
+      <c r="X27" s="11"/>
+      <c r="Y27" s="11"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="11" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B28" s="11"/>
       <c r="C28" s="11"/>
@@ -2791,10 +2894,12 @@
       <c r="U28" s="11"/>
       <c r="V28" s="11"/>
       <c r="W28" s="11"/>
+      <c r="X28" s="11"/>
+      <c r="Y28" s="11"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="11" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B29" s="11"/>
       <c r="C29" s="11"/>
@@ -2818,17 +2923,49 @@
       <c r="U29" s="11"/>
       <c r="V29" s="11"/>
       <c r="W29" s="11"/>
+      <c r="X29" s="11"/>
+      <c r="Y29" s="11"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="B30" s="11"/>
+      <c r="C30" s="11"/>
+      <c r="D30" s="11"/>
+      <c r="E30" s="11"/>
+      <c r="F30" s="11"/>
+      <c r="G30" s="11"/>
+      <c r="H30" s="11"/>
+      <c r="I30" s="11"/>
+      <c r="J30" s="11"/>
+      <c r="K30" s="11"/>
+      <c r="L30" s="11"/>
+      <c r="M30" s="11"/>
+      <c r="N30" s="11"/>
+      <c r="O30" s="11"/>
+      <c r="P30" s="11"/>
+      <c r="Q30" s="11"/>
+      <c r="R30" s="11"/>
+      <c r="S30" s="11"/>
+      <c r="T30" s="11"/>
+      <c r="U30" s="11"/>
+      <c r="V30" s="11"/>
+      <c r="W30" s="11"/>
+      <c r="X30" s="11"/>
+      <c r="Y30" s="11"/>
     </row>
   </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="A1:W1"/>
-    <mergeCell ref="A23:W23"/>
-    <mergeCell ref="A24:W24"/>
-    <mergeCell ref="A25:W25"/>
-    <mergeCell ref="A26:W26"/>
-    <mergeCell ref="A27:W27"/>
-    <mergeCell ref="A28:W28"/>
-    <mergeCell ref="A29:W29"/>
+  <mergeCells count="9">
+    <mergeCell ref="A1:Y1"/>
+    <mergeCell ref="A23:Y23"/>
+    <mergeCell ref="A24:Y24"/>
+    <mergeCell ref="A25:Y25"/>
+    <mergeCell ref="A26:Y26"/>
+    <mergeCell ref="A27:Y27"/>
+    <mergeCell ref="A28:Y28"/>
+    <mergeCell ref="A29:Y29"/>
+    <mergeCell ref="A30:Y30"/>
   </mergeCells>
   <conditionalFormatting sqref="I11:I19">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
@@ -2841,7 +2978,7 @@
       <formula>"Low Risk"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="W11:W19">
+  <conditionalFormatting sqref="Y11:Y19">
     <cfRule type="cellIs" priority="5" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
       <formula>"On Track"</formula>
     </cfRule>
@@ -2892,7 +3029,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2908,7 +3045,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -2924,7 +3061,7 @@
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="19" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B5" s="19" t="s">
         <v>26</v>
@@ -2936,28 +3073,28 @@
         <v>25</v>
       </c>
       <c r="E5" s="19" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="F5" s="19" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="G5" s="19" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="H5" s="19" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="I5" s="19" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="J5" s="19" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="K5" s="19" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="L5" s="19" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3267,7 +3404,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="11" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="B14" s="11"/>
       <c r="C14" s="11"/>
@@ -3283,7 +3420,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="B15" s="11"/>
       <c r="C15" s="11"/>
@@ -3299,7 +3436,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="11" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="B16" s="11"/>
       <c r="C16" s="11"/>
@@ -3315,7 +3452,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="11" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="B17" s="11"/>
       <c r="C17" s="11"/>
@@ -3395,7 +3532,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3415,7 +3552,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -3435,7 +3572,7 @@
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="19" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B5" s="19" t="s">
         <v>26</v>
@@ -3450,52 +3587,52 @@
         <v>25</v>
       </c>
       <c r="F5" s="19" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="G5" s="19" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="H5" s="19" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="I5" s="19" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="J5" s="19" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="K5" s="19" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="L5" s="19" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="M5" s="19" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="N5" s="19" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="O5" s="19" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="P5" s="19" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="28" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="B6" s="28" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C6" s="20" t="str">
         <f aca="false">IFERROR(INDEX('Reference Data'!$B$22:$B$27,MATCH(B6,'Reference Data'!$A$22:$A$27,0)),"N/A")</f>
         <v>Shenzhen</v>
       </c>
       <c r="D6" s="28" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="E6" s="20" t="str">
         <f aca="false">IFERROR(INDEX('Reference Data'!$B$10:$B$18,MATCH(D6,'Reference Data'!$A$10:$A$18,0)),"N/A")</f>
@@ -3505,16 +3642,16 @@
         <v>500</v>
       </c>
       <c r="G6" s="28" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="H6" s="30" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="I6" s="30" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="J6" s="28" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="K6" s="31" t="n">
         <v>5.5</v>
@@ -3542,17 +3679,17 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="28" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="B7" s="28" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C7" s="20" t="str">
         <f aca="false">IFERROR(INDEX('Reference Data'!$B$22:$B$27,MATCH(B7,'Reference Data'!$A$22:$A$27,0)),"N/A")</f>
         <v>Shenzhen</v>
       </c>
       <c r="D7" s="28" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="E7" s="20" t="str">
         <f aca="false">IFERROR(INDEX('Reference Data'!$B$10:$B$18,MATCH(D7,'Reference Data'!$A$10:$A$18,0)),"N/A")</f>
@@ -3562,16 +3699,16 @@
         <v>500</v>
       </c>
       <c r="G7" s="28" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="H7" s="30" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="I7" s="30" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="J7" s="28" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="K7" s="31" t="n">
         <v>4</v>
@@ -3599,17 +3736,17 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="28" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="B8" s="28" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="C8" s="20" t="str">
         <f aca="false">IFERROR(INDEX('Reference Data'!$B$22:$B$27,MATCH(B8,'Reference Data'!$A$22:$A$27,0)),"N/A")</f>
         <v>Jakarta</v>
       </c>
       <c r="D8" s="28" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="E8" s="20" t="str">
         <f aca="false">IFERROR(INDEX('Reference Data'!$B$10:$B$18,MATCH(D8,'Reference Data'!$A$10:$A$18,0)),"N/A")</f>
@@ -3619,19 +3756,19 @@
         <v>300</v>
       </c>
       <c r="G8" s="28" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="H8" s="30" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="I8" s="30" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="J8" s="28" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="K8" s="30" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="L8" s="32" t="str">
         <f aca="false">IFERROR(INDEX('Reference Data'!$C$31:$C$45,MATCH($C8&amp;"|"&amp;$H8,'Reference Data'!$F$31:$F$45,0)),"N/A")</f>
@@ -3656,17 +3793,17 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="28" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="B9" s="28" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="C9" s="20" t="str">
         <f aca="false">IFERROR(INDEX('Reference Data'!$B$22:$B$27,MATCH(B9,'Reference Data'!$A$22:$A$27,0)),"N/A")</f>
         <v>Taipei</v>
       </c>
       <c r="D9" s="28" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="E9" s="20" t="str">
         <f aca="false">IFERROR(INDEX('Reference Data'!$B$10:$B$18,MATCH(D9,'Reference Data'!$A$10:$A$18,0)),"N/A")</f>
@@ -3676,19 +3813,19 @@
         <v>1000</v>
       </c>
       <c r="G9" s="28" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="H9" s="30" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="I9" s="30" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="J9" s="28" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="K9" s="30" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="L9" s="32" t="str">
         <f aca="false">IFERROR(INDEX('Reference Data'!$C$31:$C$45,MATCH($C9&amp;"|"&amp;$H9,'Reference Data'!$F$31:$F$45,0)),"N/A")</f>
@@ -3713,17 +3850,17 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="28" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="B10" s="28" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="C10" s="20" t="str">
         <f aca="false">IFERROR(INDEX('Reference Data'!$B$22:$B$27,MATCH(B10,'Reference Data'!$A$22:$A$27,0)),"N/A")</f>
         <v>Chiang Mai</v>
       </c>
       <c r="D10" s="28" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="E10" s="20" t="str">
         <f aca="false">IFERROR(INDEX('Reference Data'!$B$10:$B$18,MATCH(D10,'Reference Data'!$A$10:$A$18,0)),"N/A")</f>
@@ -3733,19 +3870,19 @@
         <v>200</v>
       </c>
       <c r="G10" s="28" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="H10" s="30" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="I10" s="30" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="J10" s="28" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="K10" s="30" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="L10" s="32" t="str">
         <f aca="false">IFERROR(INDEX('Reference Data'!$C$31:$C$45,MATCH($C10&amp;"|"&amp;$H10,'Reference Data'!$F$31:$F$45,0)),"N/A")</f>
@@ -3770,17 +3907,17 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="28" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="B11" s="28" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="C11" s="20" t="str">
         <f aca="false">IFERROR(INDEX('Reference Data'!$B$22:$B$27,MATCH(B11,'Reference Data'!$A$22:$A$27,0)),"N/A")</f>
         <v>Ho Chi Minh City</v>
       </c>
       <c r="D11" s="28" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="E11" s="20" t="str">
         <f aca="false">IFERROR(INDEX('Reference Data'!$B$10:$B$18,MATCH(D11,'Reference Data'!$A$10:$A$18,0)),"N/A")</f>
@@ -3790,16 +3927,16 @@
         <v>500</v>
       </c>
       <c r="G11" s="28" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="H11" s="30" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="I11" s="30" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="J11" s="28" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="K11" s="31" t="n">
         <v>6</v>
@@ -3827,7 +3964,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="26" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B12" s="27"/>
       <c r="C12" s="27"/>
@@ -3855,7 +3992,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="B15" s="11"/>
       <c r="C15" s="11"/>
@@ -3875,7 +4012,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="11" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="B16" s="11"/>
       <c r="C16" s="11"/>
@@ -3895,7 +4032,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="11" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="B17" s="11"/>
       <c r="C17" s="11"/>
@@ -3915,7 +4052,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="11" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="B18" s="11"/>
       <c r="C18" s="11"/>
@@ -3990,7 +4127,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4009,12 +4146,12 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="12" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="B4" s="15" t="n">
         <v>4</v>
@@ -4022,13 +4159,13 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="12" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="B5" s="15" t="n">
         <v>8</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4039,40 +4176,40 @@
         <v>25</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="D7" s="19" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E7" s="19" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="F7" s="19" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="G7" s="19" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="H7" s="19" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="I7" s="19" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="J7" s="19" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="K7" s="19" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="L7" s="19" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="M7" s="19" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="N7" s="19" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="O7" s="19" t="s">
         <v>30</v>
@@ -4080,7 +4217,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="28" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="B8" s="20" t="str">
         <f aca="false">IFERROR(INDEX('Reference Data'!$B$10:$B$18,MATCH($A8,'Reference Data'!$A$10:$A$18,0)),"N/A")</f>
@@ -4137,7 +4274,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="28" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="B9" s="20" t="str">
         <f aca="false">IFERROR(INDEX('Reference Data'!$B$10:$B$18,MATCH($A9,'Reference Data'!$A$10:$A$18,0)),"N/A")</f>
@@ -4194,7 +4331,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="28" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="B10" s="20" t="str">
         <f aca="false">IFERROR(INDEX('Reference Data'!$B$10:$B$18,MATCH($A10,'Reference Data'!$A$10:$A$18,0)),"N/A")</f>
@@ -4251,7 +4388,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="28" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="B11" s="20" t="str">
         <f aca="false">IFERROR(INDEX('Reference Data'!$B$10:$B$18,MATCH($A11,'Reference Data'!$A$10:$A$18,0)),"N/A")</f>
@@ -4308,7 +4445,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="28" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="B12" s="20" t="str">
         <f aca="false">IFERROR(INDEX('Reference Data'!$B$10:$B$18,MATCH($A12,'Reference Data'!$A$10:$A$18,0)),"N/A")</f>
@@ -4365,7 +4502,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="28" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="B13" s="20" t="str">
         <f aca="false">IFERROR(INDEX('Reference Data'!$B$10:$B$18,MATCH($A13,'Reference Data'!$A$10:$A$18,0)),"N/A")</f>
@@ -4422,7 +4559,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="28" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="B14" s="20" t="str">
         <f aca="false">IFERROR(INDEX('Reference Data'!$B$10:$B$18,MATCH($A14,'Reference Data'!$A$10:$A$18,0)),"N/A")</f>
@@ -4479,7 +4616,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="28" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="B15" s="20" t="str">
         <f aca="false">IFERROR(INDEX('Reference Data'!$B$10:$B$18,MATCH($A15,'Reference Data'!$A$10:$A$18,0)),"N/A")</f>
@@ -4536,7 +4673,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="28" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="B16" s="20" t="str">
         <f aca="false">IFERROR(INDEX('Reference Data'!$B$10:$B$18,MATCH($A16,'Reference Data'!$A$10:$A$18,0)),"N/A")</f>
@@ -4593,7 +4730,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="26" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B17" s="27"/>
       <c r="C17" s="27"/>
@@ -4635,7 +4772,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="11" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="B20" s="11"/>
       <c r="C20" s="11"/>
@@ -4654,7 +4791,7 @@
     </row>
     <row r="21" customFormat="false" ht="22.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="11" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="B21" s="11"/>
       <c r="C21" s="11"/>
@@ -4673,7 +4810,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="11" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="B22" s="11"/>
       <c r="C22" s="11"/>
@@ -4692,7 +4829,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="11" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="B23" s="11"/>
       <c r="C23" s="11"/>
@@ -4769,7 +4906,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4781,7 +4918,7 @@
     </row>
     <row r="3" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
@@ -4793,51 +4930,51 @@
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="19" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="C4" s="19" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="28" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="B5" s="28" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="C5" s="28" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="28" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="B6" s="28" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="C6" s="28" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="28" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="B7" s="28" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="C7" s="28" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
@@ -4855,141 +4992,141 @@
         <v>25</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="D9" s="19" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="28" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="B10" s="28" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="C10" s="28" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="D10" s="28" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="28" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="B11" s="28" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="C11" s="28" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="D11" s="28" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="28" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="B12" s="28" t="s">
+        <v>159</v>
+      </c>
+      <c r="C12" s="28" t="s">
         <v>156</v>
       </c>
-      <c r="C12" s="28" t="s">
-        <v>153</v>
-      </c>
       <c r="D12" s="28" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="28" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="B13" s="28" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="C13" s="28" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="D13" s="28" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="28" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="B14" s="28" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="C14" s="28" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="D14" s="28" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="28" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="B15" s="28" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="C15" s="28" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="D15" s="28" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="28" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="B16" s="28" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="C16" s="28" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="D16" s="28" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="28" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="B17" s="28" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="C17" s="28" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="D17" s="28" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="28" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="B18" s="28" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="C18" s="28" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="D18" s="28" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="B20" s="3"/>
       <c r="C20" s="3"/>
@@ -5004,42 +5141,42 @@
         <v>26</v>
       </c>
       <c r="B21" s="19" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="C21" s="19" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="D21" s="19" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="E21" s="19" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="F21" s="19" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="G21" s="19" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="H21" s="19" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="28" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="B22" s="28" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="C22" s="28" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="D22" s="28" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="E22" s="28" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="F22" s="29" t="n">
         <v>500</v>
@@ -5048,24 +5185,24 @@
         <v>3</v>
       </c>
       <c r="H22" s="28" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="28" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="B23" s="28" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="C23" s="28" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="D23" s="28" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="E23" s="28" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="F23" s="29" t="n">
         <v>400</v>
@@ -5074,24 +5211,24 @@
         <v>2.5</v>
       </c>
       <c r="H23" s="28" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="28" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="B24" s="28" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="C24" s="28" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="D24" s="28" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="E24" s="28" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="F24" s="29" t="n">
         <v>300</v>
@@ -5100,24 +5237,24 @@
         <v>3</v>
       </c>
       <c r="H24" s="28" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="28" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="B25" s="28" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="C25" s="28" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="D25" s="28" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="E25" s="28" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="F25" s="29" t="n">
         <v>1000</v>
@@ -5126,24 +5263,24 @@
         <v>2</v>
       </c>
       <c r="H25" s="28" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="28" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="B26" s="28" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="C26" s="28" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="D26" s="28" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="E26" s="28" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="F26" s="29" t="n">
         <v>200</v>
@@ -5152,24 +5289,24 @@
         <v>2</v>
       </c>
       <c r="H26" s="28" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="28" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="B27" s="28" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="C27" s="28" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="D27" s="28" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="E27" s="28" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="F27" s="29" t="n">
         <v>500</v>
@@ -5178,12 +5315,12 @@
         <v>4</v>
       </c>
       <c r="H27" s="28" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="3" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="B29" s="3"/>
       <c r="C29" s="3"/>
@@ -5195,30 +5332,30 @@
     </row>
     <row r="30" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="19" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="B30" s="19" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="C30" s="19" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="D30" s="19" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="E30" s="19" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="F30" s="19" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="28" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="B31" s="28" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="C31" s="35" t="n">
         <v>3</v>
@@ -5237,10 +5374,10 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="28" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="B32" s="28" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="C32" s="35" t="n">
         <v>5</v>
@@ -5259,10 +5396,10 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="28" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="B33" s="28" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="C33" s="35" t="n">
         <v>0.285714285714286</v>
@@ -5281,10 +5418,10 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="28" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="B34" s="28" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="C34" s="35" t="n">
         <v>4.5</v>
@@ -5303,10 +5440,10 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="28" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="B35" s="28" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="C35" s="35" t="n">
         <v>4.5</v>
@@ -5325,10 +5462,10 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="28" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="B36" s="28" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="C36" s="35" t="n">
         <v>4</v>
@@ -5347,10 +5484,10 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="28" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="B37" s="28" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="C37" s="35" t="n">
         <v>4</v>
@@ -5369,10 +5506,10 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="28" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="B38" s="28" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="C38" s="35" t="n">
         <v>5</v>
@@ -5391,10 +5528,10 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="28" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="B39" s="28" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="C39" s="35" t="n">
         <v>4</v>
@@ -5413,10 +5550,10 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="28" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="B40" s="28" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="C40" s="35" t="n">
         <v>3</v>
@@ -5435,10 +5572,10 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="28" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="B41" s="28" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="C41" s="35" t="n">
         <v>5</v>
@@ -5457,10 +5594,10 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="28" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="B42" s="28" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="C42" s="35" t="n">
         <v>0.285714285714286</v>
@@ -5479,10 +5616,10 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="28" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="B43" s="28" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="C43" s="35" t="n">
         <v>3.5</v>
@@ -5501,10 +5638,10 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="28" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="B44" s="28" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="C44" s="35" t="n">
         <v>5</v>
@@ -5523,10 +5660,10 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="28" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="B45" s="28" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="C45" s="35" t="n">
         <v>3</v>
@@ -5550,7 +5687,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="11" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="B48" s="11"/>
       <c r="C48" s="11"/>
@@ -5562,7 +5699,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="11" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="B49" s="11"/>
       <c r="C49" s="11"/>
@@ -5574,7 +5711,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="11" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="B50" s="11"/>
       <c r="C50" s="11"/>
@@ -5586,7 +5723,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="11" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B51" s="11"/>
       <c r="C51" s="11"/>
@@ -5598,7 +5735,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="11" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="B52" s="11"/>
       <c r="C52" s="11"/>

</xml_diff>